<commit_message>
First working version 3D
</commit_message>
<xml_diff>
--- a/config/default/default3D.xlsx
+++ b/config/default/default3D.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="6_{21B2E60F-E45E-4B1E-BA14-FAE5B07AE4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4ABB427-BD9E-42C0-A44A-2EA8EE7E419A}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="6_{21B2E60F-E45E-4B1E-BA14-FAE5B07AE4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63444DC0-8E9C-4D4A-847F-597AEAB9D61B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="2" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
+    <workbookView xWindow="-18120" yWindow="-2550" windowWidth="18240" windowHeight="28320" activeTab="2" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="2" r:id="rId1"/>
@@ -2058,7 +2058,7 @@
         <v>49</v>
       </c>
       <c r="F5" s="11">
-        <v>1E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G5" s="29" t="s">
         <v>102</v>
@@ -2081,7 +2081,7 @@
         <v>49</v>
       </c>
       <c r="F6" s="11">
-        <v>1E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G6" s="29" t="s">
         <v>102</v>
@@ -2104,7 +2104,7 @@
         <v>49</v>
       </c>
       <c r="F7" s="11">
-        <v>5.0000000000000002E-5</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G7" s="29" t="s">
         <v>102</v>
@@ -2474,7 +2474,7 @@
         <v>101</v>
       </c>
       <c r="F5" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="G5" s="29" t="s">
         <v>102</v>
@@ -2497,7 +2497,7 @@
         <v>101</v>
       </c>
       <c r="F6" s="11">
-        <v>0.05</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="G6" s="29" t="s">
         <v>102</v>
@@ -2520,7 +2520,7 @@
         <v>101</v>
       </c>
       <c r="F7" s="11">
-        <v>2.15E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="G7" s="29" t="s">
         <v>102</v>
@@ -2543,7 +2543,7 @@
         <v>101</v>
       </c>
       <c r="F8" s="11">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="G8" s="29" t="s">
         <v>102</v>
@@ -2566,7 +2566,7 @@
         <v>101</v>
       </c>
       <c r="F9" s="11">
-        <v>0.05</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="G9" s="29" t="s">
         <v>102</v>
@@ -2589,7 +2589,7 @@
         <v>101</v>
       </c>
       <c r="F10" s="11">
-        <v>2.15E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="G10" s="29" t="s">
         <v>102</v>

</xml_diff>